<commit_message>
Docs: cover Post Builder, Google Sheet view and Draft status
README now lists all three views, the Post Builder and what the tool
doesn't do; fixes placeholder links. SETUP covers post.html in both
deploy options, the buyer sheet, and the Post Builder steps. Template
gains Draft status and the Sheet link setting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YPfDsKuCWtye1frrpJxo36
</commit_message>
<xml_diff>
--- a/template/Fragrance_Declutter_Storefront_Template.xlsx
+++ b/template/Fragrance_Declutter_Storefront_Template.xlsx
@@ -5970,7 +5970,7 @@
   </conditionalFormatting>
   <dataValidations count="5">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose Available or Sold." type="list">
-      <formula1>"Available,Sold"</formula1>
+      <formula1>"Available,Sold,Draft"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Category" error="Choose one of the three categories." type="list">
       <formula1>"Indian houses,Middle Eastern houses,Designer/Niche"</formula1>
@@ -9048,7 +9048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9241,6 +9241,14 @@
           <t>Built with Claude by Janesh S.</t>
         </is>
       </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Sheet link</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -12314,7 +12322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12383,7 +12391,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>REQUIRED. Available or Sold. Only Available items show on the website.</t>
+          <t>REQUIRED. Available, Sold or Draft. Only Available items show on the website. Use Draft for rows you are still filling in.</t>
         </is>
       </c>
     </row>
@@ -12956,12 +12964,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Discounts (D-F)</t>
+          <t>Sheet link</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Min order, Discount % (5 = 5%), Active Yes/No. The highest active tier the order reaches applies.</t>
+          <t>Optional. Link to a view-only Google Sheet of your list. When filled, a Sheet button appears next to Table and Photos. Leave blank to hide it.</t>
         </is>
       </c>
     </row>
@@ -12973,10 +12981,27 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
+          <t>Discounts (D-F)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Min order, Discount % (5 = 5%), Active Yes/No. The highest active tier the order reaches applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
           <t>Scent families (H)</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>The dropdown list for Inventory &gt; Scent Family. Add new families on the next empty row.</t>
         </is>

</xml_diff>

<commit_message>
Add sale prices: strike-through, % off badge and Sale filter
A new optional Sale Price column in Inventory. When it is below Price,
the shop shows the old price struck through, a % off badge, a Sale
filter, and uses the sale price in the cart and WhatsApp message. The
Post Builder shows it in the picker, message (~old~ new) and collages.
Apps Script passes the new column through as salePrice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YPfDsKuCWtye1frrpJxo36
</commit_message>
<xml_diff>
--- a/template/Fragrance_Declutter_Storefront_Template.xlsx
+++ b/template/Fragrance_Declutter_Storefront_Template.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:P1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,7 @@
     <col width="30" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -605,6 +606,11 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Date Listed</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Sale Price</t>
         </is>
       </c>
     </row>
@@ -12322,7 +12328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12619,17 +12625,17 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Photos</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Photo ID</t>
+          <t>Sale Price</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>A unique code for this photo. The phone app (Step 6) fills this in automatically.</t>
+          <t>Optional. A lower price for a price drop. The site strikes through Price, shows this instead with a % off badge, and lists the item under the Sale filter. Clear it to end the sale.</t>
         </is>
       </c>
     </row>
@@ -12641,12 +12647,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Item ID</t>
+          <t>Photo ID</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>The ID of the Inventory item this photo belongs to, e.g. P001.</t>
+          <t>A unique code for this photo. The phone app (Step 6) fills this in automatically.</t>
         </is>
       </c>
     </row>
@@ -12658,12 +12664,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Item ID</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>The photo file. The phone app (Step 6) saves the photo to Google Drive and fills this in.</t>
+          <t>The ID of the Inventory item this photo belongs to, e.g. P001.</t>
         </is>
       </c>
     </row>
@@ -12675,12 +12681,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Order</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>1 = cover photo (shown first), then 2, 3...</t>
+          <t>The photo file. The phone app (Step 6) saves the photo to Google Drive and fills this in.</t>
         </is>
       </c>
     </row>
@@ -12692,29 +12698,29 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Public URL</t>
+          <t>Order</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Leave blank: filled in automatically. (Advanced: you can also paste a direct image link here yourself.)</t>
+          <t>1 = cover photo (shown first), then 2, 3...</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Vouches</t>
+          <t>Photos</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Vouch ID</t>
+          <t>Public URL</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>A unique code. The phone app fills it in automatically.</t>
+          <t>Leave blank: filled in automatically. (Advanced: you can also paste a direct image link here yourself.)</t>
         </is>
       </c>
     </row>
@@ -12726,12 +12732,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Image</t>
+          <t>Vouch ID</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>A buyer's thank-you screenshot (blur names and numbers first). The phone app saves it to Drive.</t>
+          <t>A unique code. The phone app fills it in automatically.</t>
         </is>
       </c>
     </row>
@@ -12743,12 +12749,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Caption</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Optional, e.g. Pune, Lattafa set.</t>
+          <t>A buyer's thank-you screenshot (blur names and numbers first). The phone app saves it to Drive.</t>
         </is>
       </c>
     </row>
@@ -12760,12 +12766,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Caption</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Optional. Newest vouches show first.</t>
+          <t>Optional, e.g. Pune, Lattafa set.</t>
         </is>
       </c>
     </row>
@@ -12777,12 +12783,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Show</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Yes or No. No hides it from the website without deleting it.</t>
+          <t>Optional. Newest vouches show first.</t>
         </is>
       </c>
     </row>
@@ -12794,29 +12800,29 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Public URL</t>
+          <t>Show</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Leave blank: filled in automatically.</t>
+          <t>Yes or No. No hides it from the website without deleting it.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Vouches</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Store name</t>
+          <t>Public URL</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Shown at the top of the site.</t>
+          <t>Leave blank: filled in automatically.</t>
         </is>
       </c>
     </row>
@@ -12828,12 +12834,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Tagline</t>
+          <t>Store name</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Short line under the store name.</t>
+          <t>Shown at the top of the site.</t>
         </is>
       </c>
     </row>
@@ -12845,12 +12851,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp number</t>
+          <t>Tagline</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>REPLACE THIS. Country code + number, digits only, no + or spaces. Example: 919876543210</t>
+          <t>Short line under the store name.</t>
         </is>
       </c>
     </row>
@@ -12862,12 +12868,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>WhatsApp number</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Announcement strip. Clear this cell to hide the banner.</t>
+          <t>REPLACE THIS. Country code + number, digits only, no + or spaces. Example: 919876543210</t>
         </is>
       </c>
     </row>
@@ -12879,12 +12885,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Minimum order</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Rupees. Buyers below this see a warning (never blocked).</t>
+          <t>Announcement strip. Clear this cell to hide the banner.</t>
         </is>
       </c>
     </row>
@@ -12896,12 +12902,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Free shipping from</t>
+          <t>Minimum order</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Rupees. Orders under this see 'Shipping will be charged'.</t>
+          <t>Rupees. Buyers below this see a warning (never blocked).</t>
         </is>
       </c>
     </row>
@@ -12913,12 +12919,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>New badge days</t>
+          <t>Free shipping from</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Items listed within this many days get a NEW badge.</t>
+          <t>Rupees. Orders under this see 'Shipping will be charged'.</t>
         </is>
       </c>
     </row>
@@ -12930,12 +12936,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Delivery note</t>
+          <t>New badge days</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Shown in the footer.</t>
+          <t>Items listed within this many days get a NEW badge.</t>
         </is>
       </c>
     </row>
@@ -12947,12 +12953,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Credit line</t>
+          <t>Delivery note</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Shown in the footer, links to the open-source project.</t>
+          <t>Shown in the footer.</t>
         </is>
       </c>
     </row>
@@ -12964,12 +12970,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Sheet link</t>
+          <t>Credit line</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Optional. Link to a view-only Google Sheet of your list. When filled, a Sheet button appears next to Table and Photos. Leave blank to hide it.</t>
+          <t>Shown in the footer, links to the open-source project.</t>
         </is>
       </c>
     </row>
@@ -12981,12 +12987,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Discounts (D-F)</t>
+          <t>Sheet link</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Min order, Discount % (5 = 5%), Active Yes/No. The highest active tier the order reaches applies.</t>
+          <t>Optional. Link to a view-only Google Sheet of your list. When filled, a Sheet button appears next to Table and Photos. Leave blank to hide it.</t>
         </is>
       </c>
     </row>
@@ -12998,10 +13004,27 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
+          <t>Discounts (D-F)</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Min order, Discount % (5 = 5%), Active Yes/No. The highest active tier the order reaches applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
           <t>Scent families (H)</t>
         </is>
       </c>
-      <c r="C42" s="11" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>The dropdown list for Inventory &gt; Scent Family. Add new families on the next empty row.</t>
         </is>

</xml_diff>